<commit_message>
Gestion des catégories de taxe - validation livraison intracommunautaire & cas franchise de TVA
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\__dev_projects\ezfacture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D639EE8B-7886-4E23-B4D0-AB33647B917E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B1EFAD-6038-4E65-87A5-4845E2CF8227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{55AABB10-9C92-4D0A-827C-A75C8CBFF77D}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="AAB">config!$B$20</definedName>
     <definedName name="footer">config!$B$14</definedName>
-    <definedName name="liste_regimes_tva">config!$E$17:$E$18</definedName>
+    <definedName name="liste_regimes_tva">config!$E$17:$E$19</definedName>
     <definedName name="PMD">config!$B$18</definedName>
     <definedName name="PMT">config!$B$19</definedName>
     <definedName name="table_config">config!$B$2:$B$14</definedName>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
   <si>
     <t>Dénomination sociale</t>
   </si>
@@ -174,13 +174,19 @@
   </si>
   <si>
     <t>Aucun escompte accordé pour paiement anticipé</t>
+  </si>
+  <si>
+    <t>Franchise en base de TVA (art. 293 B)</t>
+  </si>
+  <si>
+    <t>Micro-entreprises</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -261,6 +267,13 @@
     <font>
       <sz val="11"/>
       <color theme="3" tint="0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.499984740745262"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -425,11 +438,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -440,6 +448,9 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
@@ -790,7 +801,7 @@
       <c r="A1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="15" t="s">
         <v>14</v>
       </c>
     </row>
@@ -798,7 +809,7 @@
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="16" t="s">
         <v>32</v>
       </c>
     </row>
@@ -806,7 +817,7 @@
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="16" t="s">
         <v>24</v>
       </c>
     </row>
@@ -814,7 +825,7 @@
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="17" t="s">
         <v>25</v>
       </c>
     </row>
@@ -822,13 +833,13 @@
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="19"/>
+      <c r="B5" s="16"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="16" t="s">
         <v>26</v>
       </c>
     </row>
@@ -836,7 +847,7 @@
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="16" t="s">
         <v>27</v>
       </c>
     </row>
@@ -844,7 +855,7 @@
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="16" t="s">
         <v>7</v>
       </c>
     </row>
@@ -852,7 +863,7 @@
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="16" t="s">
         <v>28</v>
       </c>
     </row>
@@ -860,7 +871,7 @@
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="19" t="s">
         <v>33</v>
       </c>
     </row>
@@ -868,7 +879,7 @@
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="16" t="s">
         <v>29</v>
       </c>
     </row>
@@ -876,7 +887,7 @@
       <c r="A12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="16" t="s">
         <v>30</v>
       </c>
     </row>
@@ -884,7 +895,7 @@
       <c r="A13" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="16" t="s">
         <v>31</v>
       </c>
     </row>
@@ -892,7 +903,7 @@
       <c r="A14" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="17" t="s">
         <v>34</v>
       </c>
       <c r="D14" s="6"/>
@@ -903,7 +914,7 @@
       <c r="A15" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="18" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="9" t="s">
@@ -916,7 +927,7 @@
       <c r="A16" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="18">
         <v>1</v>
       </c>
       <c r="D16" s="12" t="s">
@@ -929,7 +940,7 @@
       <c r="A17" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="18">
         <v>1</v>
       </c>
       <c r="D17" s="12"/>
@@ -944,14 +955,14 @@
       <c r="A18" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="D18" s="15"/>
-      <c r="E18" s="16" t="s">
+      <c r="D18" s="12"/>
+      <c r="E18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="14" t="s">
         <v>21</v>
       </c>
     </row>
@@ -959,15 +970,22 @@
       <c r="A19" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="20" t="s">
         <v>41</v>
+      </c>
+      <c r="D19" s="21"/>
+      <c r="E19" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="20" t="s">
         <v>42</v>
       </c>
     </row>
@@ -975,7 +993,7 @@
       <c r="A21" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="20" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>